<commit_message>
feature/fsel-6873: update delete student from curriculum
</commit_message>
<xml_diff>
--- a/Services/Fsel.Identity/Fsel.Identity.Api/Resources/Campus/StudentsInfo.xlsx
+++ b/Services/Fsel.Identity/Fsel.Identity.Api/Resources/Campus/StudentsInfo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\fsel_src\Services\Fsel.Identity\Fsel.Identity.Api\Resources\Campus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA7C2CF0-2C13-4166-A23E-584AF38CF266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F976085-61E2-4B62-837D-D1BC81AA897B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6641B693-A4D1-4DED-B7D6-AAEB74BFF851}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6641B693-A4D1-4DED-B7D6-AAEB74BFF851}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Họ và tên</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t>Mật khẩu</t>
   </si>
 </sst>
 </file>
@@ -437,10 +440,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{840462C9-2B8A-4D25-8B97-24D006999A03}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -453,6 +459,9 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>